<commit_message>
Food/Bengaluru: separate Akshayakalpa's own Meta creatives from third-party placements; rebuild pack, workbook and v3 handoff bundle
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/food-bangalore-audits/Food-Bangalore-ALL-IN-ONE.xlsx
+++ b/food-bangalore-audits/Food-Bangalore-ALL-IN-ONE.xlsx
@@ -2725,7 +2725,7 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>MEASURED — verified ad by ad</t>
+          <t>MEASURED — 3</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -4857,7 +4857,7 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Started 19 May 2026 (2 ads) · 24 Jun 2026 · 12 Aug 2026 (9 ads) · 16 Sep 2026</t>
+          <t>3 live creatives from the brand page, running since 19 May 2026 (2 creatives, 2 variants each) and 24 Jun 2026 (1 creative, 2 variants)</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
@@ -7856,7 +7856,7 @@
           <t>Hi team,
 I audit paid media for food brands from Bengaluru. Your footprint is the biggest I found in this category: ~400 live Google creatives under Akshayakalpa Farms and Foods Pvt Ltd. The product story behind it is world-class - 4C farm chilling, 24-36 hours to doorstep vs the 72-96 hour industry norm, APEDA certified.
 One thing you can check in 30 seconds: the footer of akshayakalpa.org currently contains template placeholder text - '0123.456.789 - 2 Queen Street, California, USA'. Your paid traffic lands on that page. It is a small fix and a direct trust cost while it is live.
-Attached is a 2-page audit with 3 fixes, including what I would do with ~400 creatives to make them learn faster than they spend. Worth 15 minutes?
+Attached is the 7-page Paid Media and Measurement Audit, including what I would do with ~400 creatives to make them learn faster than they spend. Worth 15 minutes?
 - Smart Pursuit, Bengaluru | 7095024220
 P.S. I am writing to your published support address because the site does not list a marketing or partner contact - that is itself one of the findings.</t>
         </is>
@@ -7992,7 +7992,7 @@
           <t>Hi team,
 I run paid-media audits for Bengaluru food brands. I checked your live footprint: 58 Google creatives under Anand Sweets &amp; Savouries LLP, and Google shows you as a Verified advertiser - a real asset in mithai, where trust decides the order.
 The problem: your own top banner tells every paid visitor that Bangalore delivery takes up to 3 days and sends same-day buyers to Swiggy, Zomato or Ownly. That is the exact moment - festive, urgent, gift-driven - where mithai margins live, and it is being handed to an aggregator.
-Attached is a 2-page audit with 3 fixes. Open to a 15-minute call?
+Attached is the 7-page Paid Media and Measurement Audit. Open to a 15-minute call?
 - Smart Pursuit, Bengaluru | 7095024220</t>
         </is>
       </c>
@@ -8127,7 +8127,7 @@
           <t>Hi team,
 I run paid-media audits for food brands from Bengaluru. I checked your live presence this week: Milky Mist Dairy Food Limited shows 3 live Google creatives - while the corporate site carries a full IPO section, SEBI Reg 46 disclosures and investor pages.
 That gap matters now: paneer, curd, ghee and cheese searches are high-intent purchase moments, and today they are being answered by Amul, Nandini and quick-commerce private labels. Before a listing, demand durability is part of the story you will be asked about.
-Attached is a 2-page audit with 3 fixes. Open to 15 minutes?
+Attached is the 7-page Paid Media and Measurement Audit. Open to 15 minutes?
 - Smart Pursuit, Bengaluru | 7095024220</t>
         </is>
       </c>
@@ -8262,7 +8262,7 @@
           <t>Hi team,
 I run paid-media audits for food brands from Bengaluru. I checked your live footprint this week: Google Ads Transparency shows one live creative for idfreshfood.com, running under Blink Digital India Pvt Ltd.
 That is remarkable for a brand at INR 681 Cr revenue with an IPO in view - and it means every 'idli batter home delivery', 'malabar parota online' or 'preservative-free batter' search is being answered by quick-commerce and smaller D2C brands, not by you.
-I have attached a 2-page audit with 3 fixes, including the subscription engine that would add recurring revenue before your IPO window. 15 minutes this week?
+I have attached the 7-page Paid Media and Measurement Audit, including the subscription engine that would add recurring revenue before your IPO window. 15 minutes this week?
 - Smart Pursuit, Bengaluru | 7095024220</t>
         </is>
       </c>
@@ -8397,7 +8397,7 @@
           <t>Hi team,
 I audit paid media for Bengaluru food brands. I checked your live footprint: 56 Google creatives under Mountain Trail Foods, a genuinely modern site (GA4 G-EN77D2S0YH), and the numbers you publish are strong - 150+ stores, 900,000 cups a day, 8,100 workplace clients.
 Here is the leak: the B2B side - your highest-value line - has no paid funnel. No 'book a demo' path for office admins searching for tea vending, while your Brewing Bot (real tea leaves, not premix) is a genuinely superior product to every coffee-only incumbent.
-Attached: a 2-page audit with 3 fixes. Worth 15 minutes?
+Attached: the 7-page Paid Media and Measurement Audit. Worth 15 minutes?
 - Smart Pursuit, Bengaluru | 7095024220</t>
         </is>
       </c>
@@ -8531,7 +8531,7 @@
           <t>Hi team,
 I audit paid media for Bengaluru food brands. I inspected your live footprint this week: 77 Google creatives running under Freeflow Creative Services, including Local store ads like your HMT Road Mathikere store. Genuinely good work - most heritage brands your age run zero paid.
 The gap: a cafe owner searching 'coffee vending machine', a household buying filter coffee, and someone near a CoCo outlet all land on the same destination. Three buyers, one page.
-Attachment: a 2-page audit with 3 fixes. Worth a short call?
+Attachment: the 7-page Paid Media and Measurement Audit. Worth a short call?
 - Smart Pursuit, Bengaluru | 7095024220</t>
         </is>
       </c>
@@ -8666,7 +8666,7 @@
           <t>Hi team,
 I audit paid media for Bengaluru food brands. I checked your live footprint: 30 Google creatives under Early Foods Pvt Ltd, plus a global storefront already live - strong setup for a clean-label brand.
 One finding: in baby food, parents are not choosing between brands - they are weighing the risk of trying you against a known multinational. Your ads and landing path lead with product; they should lead with reassurance: age-appropriate, full ingredient list, what is NOT inside, and other parents' faces.
-Attached: a 2-page audit with 3 fixes. Open to 15 minutes?
+Attached: the 7-page Paid Media and Measurement Audit. Open to 15 minutes?
 - Smart Pursuit, Bengaluru | 7095024220</t>
         </is>
       </c>
@@ -8802,7 +8802,7 @@
           <t>Hi team,
 I run paid-media audits for food brands out of Bengaluru. Over the last few days I inspected your live ad footprint - not a guess: Google Ads Transparency shows ~300 creatives under Delightful Gourmet Pvt Ltd, and I verified your Meta flight live in the Ad Library (Library ID 983369480870934, running since 15 Apr 2026).
 One finding you can act on today: that live Meta ad sends Bengaluru clicks to licious.in/store-locator. Buyers who tapped because of 'never frozen' arrive at a city picker - one full step before they see a product or price.
-I have attached a 2-page audit with 3 fixes, all doable without increasing spend. Worth 15 minutes?
+I have attached the 7-page Paid Media and Measurement Audit, all doable without increasing spend. Worth 15 minutes?
 - Smart Pursuit, Bengaluru | 7095024220
 P.S. The 0-4C cold-chain story is genuinely your strongest asset. It deserves to be the hero of the landing page, not just the ad.</t>
         </is>
@@ -8938,7 +8938,7 @@
           <t>Hi team,
 I run paid-media audits for food brands from Bengaluru. I inspected your live footprint: 35 Google creatives under Mimansa Industries Pvt Ltd - and 1M+ sourdoughs baked, which is the strongest trust proof in Indian sourdough.
 The leak: your paid clicks do not land on a 'where is my nearest loaf' page. For a brand in 300+ cities with quick-commerce distribution, that question is the whole conversion. The buyer asks it, does not get one-tap answer, and the aggregator keeps the relationship.
-Attached is a 2-page audit with 3 fixes. Open to a short call?
+Attached is the 7-page Paid Media and Measurement Audit. Open to a short call?
 - Smart Pursuit, Bengaluru | 7095024220</t>
         </is>
       </c>
@@ -9073,7 +9073,7 @@
           <t>Hi team,
 I audit paid media for Bengaluru food brands. I checked Google Ads Transparency for your domain this week and found zero live creatives - verified, on the Google side.
 For a brand with USD 112M raised and ~100 outlets, that means every 'coffee near me', 'cold brew delivery' and 'coffee beans online' query in your cities is answered by competitors. Local store campaigns are the cheapest walk-in channel a cafe chain can buy.
-I have attached a 2-page audit with 3 fixes, starting with the one I would run this month. To be clear about scope: this audit verifies Google - I have not claimed anything about your Meta inventory. Open to 15 minutes?
+I have attached the 7-page Paid Media and Measurement Audit, starting with the one I would run this month. To be clear about scope: this audit verifies Google - I have not claimed anything about your Meta inventory. Open to 15 minutes?
 - Smart Pursuit, Bengaluru | 7095024220</t>
         </is>
       </c>
@@ -9208,7 +9208,7 @@
 I audit paid media for Bengaluru food brands. I checked your live footprint: 11 Google creatives under Munchbox Frozen Foods Pvt Ltd, plus two brands (Frozen Bottle and Lubov Patisserie) and a franchise model with city and master-franchise pages.
 The gap: a single franchise sale is worth lakhs and the investor researches online first - but there is no structured paid funnel for franchise enquiries, and no store-radius campaigns for the outlets. Both are cheap to run and easy to measure.
 One small thing you can fix today: the footer links to /pages/faqs, but /pages/faq returns a 404.
-Attached is a 2-page audit with 3 fixes. Worth 15 minutes?
+Attached is the 7-page Paid Media and Measurement Audit. Worth 15 minutes?
 - Smart Pursuit, Bengaluru | 7095024220</t>
         </is>
       </c>
@@ -13908,9 +13908,10 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>meta ads:   live — running since 19 May 2026, 24 Jun 2026, 12 Aug 2026, 16 Sep 2026
-site root:  no meta pixel selector resolved on the crawl
-method:     single-method result — not asserted as absence</t>
+          <t>meta ads:    3 live creatives from the brand page (19 May and 24 Jun 2026)
+third-party:  Swiggy Instamart creative, 9 variants (12 Aug 2026)
+site root:   no meta pixel selector resolved on the crawl
+method:      single-method result — not asserted as absence</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -13940,9 +13941,9 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>creative observed:  Swiggy Instamart — organic protein, Insta-delivered
+          <t>creative observed:  Swiggy Instamart — Akshayakalpa paneer, 9 variants (12 Aug 2026)
 creative observed:  Zepto — quick-commerce placements under the term
-brand account:       separate creatives, running since May–Sep 2026</t>
+brand page:         3 creatives, running since 19 May 2026</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Food/Bengaluru: add VERIFY-THE-DATA.md verification guide (49 claim-to-source rows) + 'Verify These (links)' and 'Cannot be verified' Excel sheets; correct Akshayakalpa placeholder location to the Contact Us page and reframe the Frozen Bottle stale URL finding precisely
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/food-bangalore-audits/Food-Bangalore-ALL-IN-ONE.xlsx
+++ b/food-bangalore-audits/Food-Bangalore-ALL-IN-ONE.xlsx
@@ -19,12 +19,15 @@
     <sheet name="Opportunity Score" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Coverage (measured vs not)" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Evidence Register" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Verify These (links)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Cannot be verified" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Leads'!$A$1:$O$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Emails'!$A$1:$F$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Findings (severity+evidence)'!$A$1:$F$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Evidence Register'!$A$1:$E$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Verify These (links)'!$A$1:$E$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +62,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="001155CC"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="11">
@@ -140,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -176,6 +184,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -904,7 +915,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Placeholder international contact block on an India-facing site.</t>
+          <t>Placeholder international contact block on the Contact Us page.</t>
         </is>
       </c>
       <c r="E4" s="6" t="n">
@@ -2492,7 +2503,7 @@
         </is>
       </c>
       <c r="E52" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
@@ -2517,15 +2528,15 @@
         </is>
       </c>
       <c r="C53" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Small live footprint; conversion path has a broken page.</t>
+          <t>Small live footprint; a stale FAQ URL and an unconfigured 404 template.</t>
         </is>
       </c>
       <c r="E53" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
@@ -2558,7 +2569,7 @@
         </is>
       </c>
       <c r="E54" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
@@ -2587,11 +2598,11 @@
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Standard Shopify stack; one broken page observed.</t>
+          <t>Standard Shopify stack; stale URL variant and placeholder 404 template.</t>
         </is>
       </c>
       <c r="E55" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
@@ -2624,7 +2635,7 @@
         </is>
       </c>
       <c r="E56" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
@@ -6893,6 +6904,1523 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:E78"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="72" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Claim in the audit</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Where to check it</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>What you should see</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Akshayakalpa Organic</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>≈400 live Google creatives</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Google Ads Transparency Center (region: India)</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>https://adstransparency.google.com/?region=IN&amp;domain=akshayakalpa.org</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Around 400 creatives — the largest paid footprint in this set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Akshayakalpa Organic</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>3 live Meta creatives from the brand page</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Meta Ad Library (country: India)</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?active_status=active&amp;ad_type=all&amp;country=IN&amp;q=Akshayakalpa&amp;search_type=keyword_unordered</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Three creatives from the Akshayakalpa page; the audit cites their running-since dates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Akshayakalpa Organic</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Meta IDs 2186726058790625 · 935934206094801 · 958522520368361</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Meta Ad Library — individual ads</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=935934206094801</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Opens the creative running since 19 May 2026. Swap the id for either of the other two.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Akshayakalpa Organic</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Swiggy Instamart runs Akshayakalpa product creative</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Meta Ad Library</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=3384075765110108</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>A Swiggy Instamart placement featuring Akshayakalpa paneer, 9 variants. This is third-party distribution, not the brand's own account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Akshayakalpa Organic</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Contact Us page shows '0123.456.789 - 2 Queen Street, California'</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>akshayakalpa.org/contact-us</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>https://akshayakalpa.org/contact-us</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>The placeholder text sits at the top of the Contact Us page. Note the contrast: the homepage footer carries the correct Tiptur, Karnataka address, which is why the audit names the exact page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Akshayakalpa Organic</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>No cache-control, no HSTS</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Response headers of akshayakalpa.org</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>https://securityheaders.com/?q=akshayakalpa.org</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Or from a terminal: curl -I https://akshayakalpa.org — neither header comes back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Akshayakalpa Organic</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>support@akshayakalpa.org</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>akshayakalpa.org FAQ and privacy policy</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>https://akshayakalpa.org/</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>The only official address the brand publishes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Anand Sweets</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>58 live Google creatives</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Google Ads Transparency Center (region: India)</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>https://adstransparency.google.com/?region=IN&amp;domain=anandsweets.in</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Around 58 creatives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Anand Sweets</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>OpenAI ads pixel MsnBMqKgkHz42jqdSfTfFQ</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>anandsweets.in page source</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>https://anandsweets.in</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Ctrl+U then Ctrl+F 'MsnBMqKgkHz42jqdSfTfFQ' — the OpenAI advertising pixel is in the storefront source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Anand Sweets</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>HSTS, CSP, X-Frame-Options all present</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Response headers</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>https://securityheaders.com/?q=anandsweets.in</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>All four header families return a pass — the strongest posture in this set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Anand Sweets</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>4.4 rating from 250 reviews</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>anandsweets.in structured data</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>https://anandsweets.in</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Ctrl+F 'aggregateRating' in the page source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Anand Sweets</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>care@anandsweets.net</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>anandsweets.in footer / contact</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>https://www.anandsweets.in/</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Published in the site footer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Milky Mist</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>3 live Google creatives</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Google Ads Transparency Center (region: India)</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>https://adstransparency.google.com/?region=IN&amp;domain=milkymist.com</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Around 3 creatives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Milky Mist</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Wix behind Varnish</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Response headers</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>https://securityheaders.com/?q=milkymist.com</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Server headers show Varnish and Wix identifiers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Milky Mist</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>customercare@milkymist.com</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>milkymist.com/reach-us</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>https://milkymist.com/reach-us</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Published on the reach-us page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>iD Fresh Food</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>1 live Google creative</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Google Ads Transparency Center (region: India)</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>https://adstransparency.google.com/?region=IN&amp;domain=idfreshfood.com</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>A single creative — the finding that drives this audit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>iD Fresh Food</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Access-Control-Allow-Origin: *</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Response headers</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>https://securityheaders.com/?q=idfreshfood.com</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Or: curl -I https://idfreshfood.com — the wildcard CORS header is returned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>iD Fresh Food</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>LiteSpeed cache HIT</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Response headers</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>https://securityheaders.com/?q=idfreshfood.com</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>The cache header reports a hit, confirming the cache layer works.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>iD Fresh Food</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>customercare@idfreshfood.com</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>idfreshfood.com/contact-us</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>https://idfreshfood.com/contact-us</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Published on the contact page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>iD Fresh Food</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>FY25 revenue ≈Rs 681.4 Cr, PAT ≈Rs 25.87 Cr</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Published FY25 results as reported</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>https://idfreshfood.com/</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Figures are quoted as reported, not audited by us.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Chai Point</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>56 live Google creatives</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Google Ads Transparency Center (region: India)</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>https://adstransparency.google.com/?region=IN&amp;domain=chaipoint.com</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Around 56 creatives, under Mountain Trail Foods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Chai Point</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>GA4 G-EN77D2S0YH on the site root</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>chaipoint.com page source</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>https://chaipoint.com</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Ctrl+U then Ctrl+F 'G-EN77D2S0YH'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Chai Point</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>900,000+ cups a day · 150+ stores · 8,100+ workplaces</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>chaipoint.com structured data (JSON-LD)</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>https://chaipoint.com</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Ctrl+F 'cups' or '900' in the page source; the figures are in the machine-readable JSON-LD block.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Chai Point</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Static build on Amazon S3 + CloudFront</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Response headers</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>https://securityheaders.com/?q=chaipoint.com</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Server headers show cloudfront and S3 asset hosting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Chai Point</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>customercare@chaipoint.com</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Chai Point help centre</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>https://shop.chaipoint.com/</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Published on the order site's help section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Cothas Coffee</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>77 live Google creatives</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Google Ads Transparency Center (region: India)</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>https://adstransparency.google.com/?region=IN&amp;domain=cothas.com</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Around 77 creatives, under Freeflow Creative Services.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Cothas Coffee</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Tag layer unconfirmed</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Chrome DevTools on cothas.com</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>https://cothas.com</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>This is the one claim you can settle in a browser: open DevTools → Network, filter 'collect' or 'gtm', and reload. If tags fire, the audit's 'unconfirmed' wording is exactly right — and the fix is simply to confirm it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Cothas Coffee</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>customercare@cothas.com</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>cothas.com/pages/contact-us</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>https://cothas.com/pages/contact-us</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>Published on the contact page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Cothas Coffee</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Founded 1948, Jigani facility</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Cothas Coffee — own pages</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>https://cothas.com/</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Stated on the brand's own site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Early Foods</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>30 live Google creatives</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Google Ads Transparency Center (region: India)</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>https://adstransparency.google.com/?region=IN&amp;domain=earlyfoods.com</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>Around 30 creatives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Early Foods</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Shopify theme 124761112618 behind Cloudflare</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Response headers + page source</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>https://earlyfoods.com</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Cloudflare reported in the server headers; the theme ID appears in the storefront source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Early Foods</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>hello@earlyfoods.com</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>earlyfoods.com</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>https://earlyfoods.com/</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Published on the site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Licious</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>≈300 live Google creatives</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Google Ads Transparency Center (region: India)</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>https://adstransparency.google.com/?region=IN&amp;domain=licious.in</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>The page header reads approximately 300 ads, under Delightful Gourmet Pvt Ltd (Verified).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Licious</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>≈550 live Meta ads</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Meta Ad Library (country: India)</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?active_status=active&amp;ad_type=all&amp;country=IN&amp;q=Licious&amp;search_type=keyword_unordered</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>Around 550 results for the brand term.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Licious</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Meta library ID 983369480870934</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Meta Ad Library — the ad itself</t>
+        </is>
+      </c>
+      <c r="D36" s="15" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ads/library/?id=983369480870934</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>The specific Licious ad referenced in the audit, with its running-since date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Licious</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>GTM-KVBCJN · GA4 G-YN0TX18PEE · Ads AW-871318622</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>licious.in page source</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>https://licious.in</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Open the page, press Ctrl+U (view source), then Ctrl+F each ID. All four appear, including Meta pixel 378591842535023.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Licious</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>FY25 revenue ≈Rs 795 Cr, loss ≈Rs 218.3 Cr</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>licious.in — published company results</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
+        <is>
+          <t>https://www.licious.in/</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>Published in the company's reported FY25 results. This is a third-party reported figure, quoted as reported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Licious</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>talktous@licious.com</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>licious.in support / contact page</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>https://www.licious.in/</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Publish in the site's contact or help section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>The Baker's Dozen</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>35 live Google creatives</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Google Ads Transparency Center (region: India)</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>https://adstransparency.google.com/?region=IN&amp;domain=thebakersdozen.in</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Around 35 creatives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>The Baker's Dozen</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>GTM-MQQF2MXB · Ads AW-618150299</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>thebakersdozen.in page source</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>https://thebakersdozen.in</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Ctrl+F each ID in the page source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>The Baker's Dozen</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Meta pixel 3996239487069441</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>thebakersdozen.in page source</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>https://thebakersdozen.in</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Ctrl+F '3996239487069441'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>The Baker's Dozen</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>No HSTS, no cache-control, no security headers</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Response headers</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>https://securityheaders.com/?q=thebakersdozen.in</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>Most or all headers return a fail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>The Baker's Dozen</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>fresh@thebakersdozen.in</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>thebakersdozen.in/contact-us</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>https://thebakersdozen.in/contact-us</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>Published on the contact page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Third Wave Coffee</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Title tag is the domain string</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>thirdwavecoffeeroasters.com page source</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>https://thirdwavecoffeeroasters.com</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>Ctrl+U and look at the first line inside &lt;head&gt;: the title reads 'www.thirdwavecoffeeroasters.com' instead of the brand name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Third Wave Coffee</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>0 live Google creatives</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Google Ads Transparency Center (region: India)</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>https://adstransparency.google.com/?region=IN&amp;domain=thirdwavecoffeeroasters.com</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>No creatives are returned for the domain. The audit states this as measured on one day for this domain, not as a claim about the whole account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Third Wave Coffee</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>orders@thirdwavecoffee.in</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>thirdwavecoffee.in/pages/contact</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>https://thirdwavecoffee.in/pages/contact</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>Published on the contact page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Frozen Bottle</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>11 live Google creatives</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>Google Ads Transparency Center (region: India)</t>
+        </is>
+      </c>
+      <c r="D48" s="15" t="inlineStr">
+        <is>
+          <t>https://adstransparency.google.com/?region=IN&amp;domain=frozenbottle.com</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>Around 11 creatives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>Frozen Bottle</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>A stale FAQ URL returns 404</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>frozenbottle.com/pages/faq vs the live /pages/faqs</t>
+        </is>
+      </c>
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>https://frozenbottle.com/pages/faq</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>The singular URL returns 'not found'. The working FAQ is the plural one: frozenbottle.com/pages/faqs — the audit states both, so you can see exactly what is and is not broken.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>Frozen Bottle</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>vipul@frozenbottle.in</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>frozenbottle.com footer (partnership section)</t>
+        </is>
+      </c>
+      <c r="D50" s="15" t="inlineStr">
+        <is>
+          <t>https://frozenbottle.com/</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>Published under collaboration and partnership in the footer.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E50"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId49"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Why no public source exists</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Ad spend (Rs/month)</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>No public source exists. Ad platforms do not disclose spend for commercial advertisers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>ROAS and CPA</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Only visible inside the advertiser's own ad accounts and analytics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Conversion rates</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Private to the advertiser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Internal revenue splits by channel</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Private to the advertiser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr"/>
+      <c r="B6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Rule applied in every audit</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Where a value could not be measured it is reported as unavailable or not measured. Nothing has been inferred to fill a gap, and no tag is described as absent unless a second method confirmed it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7855,7 +9383,7 @@
         <is>
           <t>Hi team,
 I audit paid media for food brands from Bengaluru. Your footprint is the biggest I found in this category: ~400 live Google creatives under Akshayakalpa Farms and Foods Pvt Ltd. The product story behind it is world-class - 4C farm chilling, 24-36 hours to doorstep vs the 72-96 hour industry norm, APEDA certified.
-One thing you can check in 30 seconds: the footer of akshayakalpa.org currently contains template placeholder text - '0123.456.789 - 2 Queen Street, California, USA'. Your paid traffic lands on that page. It is a small fix and a direct trust cost while it is live.
+One thing you can check in 30 seconds: the Contact Us page at akshayakalpa.org/contact-us currently contains template placeholder text - '0123.456.789 - 2 Queen Street, California, USA'. Your paid traffic lands on that page. It is a small fix and a direct trust cost while it is live.
 Attached is the 7-page Paid Media and Measurement Audit, including what I would do with ~400 creatives to make them learn faster than they spend. Worth 15 minutes?
 - Smart Pursuit, Bengaluru | 7095024220
 P.S. I am writing to your published support address because the site does not list a marketing or partner contact - that is itself one of the findings.</t>
@@ -9402,7 +10930,7 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Live footer template text - '0123.456.789 - 2 Queen Street, California, USA' - sits on the pages paid traffic lands on. Small fix, direct trust cost while live.</t>
+          <t>Live Contact Us template text - '0123.456.789 - 2 Queen Street, California, USA' - sits on a page paid traffic can land on. Small fix, direct trust cost while live.</t>
         </is>
       </c>
     </row>
@@ -12247,7 +13775,7 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Placeholder footer live</t>
+          <t>Placeholder contact block live</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -13148,7 +14676,7 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>akshayakalpa.org (FAQ, company, privacy policy, contact pages): 4C farm chilling, 24-36 hr delivery claim, APEDA + Jaivik Bharat certification, farm locations, support@akshayakalpa.org / +91-9535388122, and live footer placeholder text.</t>
+          <t>akshayakalpa.org (FAQ, company, privacy policy, contact pages): 4C farm chilling, 24-36 hr delivery claim, APEDA + Jaivik Bharat certification, farm locations, support@akshayakalpa.org / +91-9535388122, and live Contact Us page placeholder text.</t>
         </is>
       </c>
     </row>
@@ -13838,19 +15366,19 @@
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>The site footer carries an international placeholder phone number and address</t>
+          <t>The Contact Us page carries an international template placeholder</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>footer text:  0123.456.789 – 2 Queen Street, California
-site:        akshayakalpa.org (India-facing)
-published:   Tiptur farms, Karnataka; corporate office Bengaluru</t>
+          <t>page:      akshayakalpa.org/contact-us
+text:      "0123.456.789 - 2 Queen Street,California, USA"
+homepage:  correct Tiptur, Karnataka address published</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>A placeholder contact block on a site taking dairy subscriptions actively damages trust and is trivially fixable. Every other finding in this report is secondary to it.</t>
+          <t>The Contact Us page a paid visitor can reach still shows a US placeholder phone number and address, while the site footer shows the correct Tiptur address. On a site selling dairy subscriptions, that inconsistency costs trust and takes minutes to correct.</t>
         </is>
       </c>
     </row>
@@ -15457,19 +16985,18 @@
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>The FAQ page returns a 404 error</t>
+          <t>Eleven live creatives is below the learning threshold for this category</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>url:    frozenbottle.com/pages/faq
-status: HTTP 404
-context: linked from the storefront navigation</t>
+          <t>google creatives live: ≈11 (region India)
+category:              desserts, ice cream and gifting</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>Frequently-asked questions are where dessert and gifting customers resolve delivery doubts. A dead page is a lost order, and on Shopify it is usually a two-minute fix.</t>
+          <t>Eleven creatives across any meaningful audience set will not separate creative from audience effects. Two clean tests would tell more than eleven undifferentiated ads.</t>
         </is>
       </c>
     </row>
@@ -15482,25 +17009,27 @@
       <c r="B54" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="C54" s="12" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Eleven live creatives is below the learning threshold for this category</t>
+          <t>A stale FAQ URL returns 404, and the 404 template still shows placeholder products</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>google creatives live: ≈11 (region India)
-category:              desserts, ice cream and gifting</t>
+          <t>url:           frozenbottle.com/pages/faq → HTTP 404
+live FAQ:      frozenbottle.com/pages/faqs (plural) works
+404 template:  'Example product $29' cards still render
+homepage:      links only to the working plural URL</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>Eleven creatives across any meaningful audience set will not separate creative from audience effects. Two clean tests would tell more than eleven undifferentiated ads.</t>
+          <t>The live FAQ is reachable, so no customer is blocked today. What remains is a stale URL that should redirect to the working one, and a 404 template still showing unconfigured Shopify placeholder cards. Both are minutes of theme work, and both are visible the moment a paid visitor mistypes a link.</t>
         </is>
       </c>
     </row>

</xml_diff>